<commit_message>
docs(hardware): update bill of materials
</commit_message>
<xml_diff>
--- a/Hardware/BOM/BOM.xlsx
+++ b/Hardware/BOM/BOM.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zoe\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zoe\Documents\PlatformIO\Projects\CodexLight\Hardware\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD3B3DBB-7066-455B-B22A-C0E535BD6046}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FF9BF4D-E3D3-4007-870C-BC0F6891464E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -129,9 +129,6 @@
     <t>MX1.25 BAT</t>
   </si>
   <si>
-    <t>CONN-SMD_2P-P1.25_XUNPU_WAFER-MX1.25-2PWB</t>
-  </si>
-  <si>
     <t>BAT1</t>
   </si>
   <si>
@@ -154,6 +151,10 @@
   </si>
   <si>
     <t>1x8P</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MX1.25 Battery-601015</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -244,23 +245,23 @@
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -545,283 +546,283 @@
   <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9" style="3"/>
-    <col min="2" max="2" width="18.375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="27.25" style="3" customWidth="1"/>
-    <col min="4" max="4" width="11.875" style="3" customWidth="1"/>
-    <col min="5" max="16384" width="9" style="3"/>
+    <col min="1" max="1" width="9" style="2"/>
+    <col min="2" max="2" width="18.375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="27.25" style="2" customWidth="1"/>
+    <col min="4" max="4" width="11.875" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="2" t="s">
+      <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="18.75" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" s="6" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="5">
-        <v>1</v>
-      </c>
-      <c r="B3" s="5" t="s">
+    <row r="3" spans="1:5" s="4" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="5">
-        <v>1</v>
-      </c>
-      <c r="E3" s="5" t="s">
+      <c r="D3" s="3">
+        <v>1</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" s="6" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="5">
+    <row r="4" spans="1:5" s="4" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="3">
         <v>3</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" s="6" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="5">
+    <row r="5" spans="1:5" s="4" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="3">
         <v>3</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:5" s="6" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="5">
+    <row r="6" spans="1:5" s="4" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3">
         <v>4</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="5">
-        <v>1</v>
-      </c>
-      <c r="E6" s="5" t="s">
+      <c r="D6" s="3">
+        <v>1</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:5" s="6" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="5">
+    <row r="7" spans="1:5" s="4" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3">
         <v>5</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="3">
         <v>5050</v>
       </c>
-      <c r="D7" s="5">
-        <v>1</v>
-      </c>
-      <c r="E7" s="5" t="s">
+      <c r="D7" s="3">
+        <v>1</v>
+      </c>
+      <c r="E7" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:5" s="6" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="5">
+    <row r="8" spans="1:5" s="4" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="3">
         <v>6</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="3">
         <v>5050</v>
       </c>
-      <c r="D8" s="5">
-        <v>1</v>
-      </c>
-      <c r="E8" s="5" t="s">
+      <c r="D8" s="3">
+        <v>1</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:5" s="6" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="5">
+    <row r="9" spans="1:5" s="4" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3">
         <v>7</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="5">
-        <v>1</v>
-      </c>
-      <c r="E9" s="5" t="s">
+      <c r="D9" s="3">
+        <v>1</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:5" s="6" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="5">
+    <row r="10" spans="1:5" s="4" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3">
         <v>8</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="3">
         <v>2</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:5" s="6" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="5">
+    <row r="11" spans="1:5" s="4" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="3">
         <v>9</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="3">
+        <v>1</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" s="4" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
+        <v>10</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="3">
+        <v>1</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" s="4" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3">
+        <v>11</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D11" s="5">
-        <v>1</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" s="6" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="5">
-        <v>10</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="5">
-        <v>1</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" s="6" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="5">
-        <v>11</v>
-      </c>
-      <c r="B13" s="5" t="s">
+      <c r="D13" s="3">
+        <v>2</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" s="4" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3">
+        <v>12</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="3">
+        <v>5050</v>
+      </c>
+      <c r="D14" s="3">
+        <v>1</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" s="4" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="3">
+        <v>13</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C13" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="D13" s="5">
+      <c r="D15" s="3">
+        <v>1</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" s="4" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3">
+        <v>14</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D16" s="3">
         <v>2</v>
       </c>
-      <c r="E13" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" s="6" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="5">
-        <v>12</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14" s="5">
-        <v>5050</v>
-      </c>
-      <c r="D14" s="5">
-        <v>1</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" s="6" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="5">
-        <v>13</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D15" s="5">
-        <v>1</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" s="6" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="5">
-        <v>14</v>
-      </c>
-      <c r="B16" s="5" t="s">
+      <c r="E16" s="3" t="s">
         <v>36</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="D16" s="5">
-        <v>2</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>